<commit_message>
feat: Implement whole number display for Excel scores and enhance numeric formatting
</commit_message>
<xml_diff>
--- a/SAMPLE_Compact_Exam_Export.xlsx
+++ b/SAMPLE_Compact_Exam_Export.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IT101 - A" sheetId="1" r:id="R3095ab4e89484746"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IT101 - A" sheetId="1" r:id="Re944d5bf41964992"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13,6 +13,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:numFmts count="1">
+    <x:numFmt numFmtId="200" formatCode="0"/>
+  </x:numFmts>
   <x:fonts count="5">
     <x:font>
       <x:sz val="11"/>
@@ -97,7 +100,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="63">
+  <x:cellXfs count="69">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -233,6 +236,22 @@
       <x:alignment horizontal="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="3" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="4" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
     </x:xf>
   </x:cellXfs>
@@ -480,22 +499,22 @@
       <x:c r="B2" s="50" t="str">
         <x:v>Ana Reyes</x:v>
       </x:c>
-      <x:c r="C2" s="46" t="n">
+      <x:c r="C2" s="64" t="n">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="D2" s="46" t="n">
+      <x:c r="D2" s="64" t="n">
         <x:v>75</x:v>
       </x:c>
-      <x:c r="E2" s="46" t="n">
+      <x:c r="E2" s="64" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="F2" s="46" t="n">
+      <x:c r="F2" s="64" t="n">
         <x:v>54</x:v>
       </x:c>
-      <x:c r="G2" s="46" t="n">
+      <x:c r="G2" s="64" t="n">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="H2" s="55" t="n">
+      <x:c r="H2" s="65" t="n">
         <x:f>SUM(C2:F2)</x:f>
         <x:v>169</x:v>
       </x:c>
@@ -507,16 +526,16 @@
       <x:c r="B3" s="51" t="str">
         <x:v>Ben Santos</x:v>
       </x:c>
-      <x:c r="C3" s="47" t="n">
+      <x:c r="C3" s="66" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D3" s="58"/>
-      <x:c r="E3" s="58"/>
-      <x:c r="F3" s="58"/>
-      <x:c r="G3" s="47" t="n">
+      <x:c r="D3" s="67"/>
+      <x:c r="E3" s="67"/>
+      <x:c r="F3" s="67"/>
+      <x:c r="G3" s="66" t="n">
         <x:v>18</x:v>
       </x:c>
-      <x:c r="H3" s="62" t="n">
+      <x:c r="H3" s="68" t="n">
         <x:f>SUM(C3:F3)</x:f>
         <x:v>0</x:v>
       </x:c>
@@ -528,22 +547,22 @@
       <x:c r="B4" s="50" t="str">
         <x:v>Cara Lim</x:v>
       </x:c>
-      <x:c r="C4" s="46" t="n">
+      <x:c r="C4" s="64" t="n">
         <x:v>48</x:v>
       </x:c>
-      <x:c r="D4" s="46" t="n">
+      <x:c r="D4" s="64" t="n">
         <x:v>88</x:v>
       </x:c>
-      <x:c r="E4" s="46" t="n">
+      <x:c r="E4" s="64" t="n">
         <x:v>37</x:v>
       </x:c>
-      <x:c r="F4" s="46" t="n">
+      <x:c r="F4" s="64" t="n">
         <x:v>58</x:v>
       </x:c>
-      <x:c r="G4" s="46" t="n">
+      <x:c r="G4" s="64" t="n">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="H4" s="55" t="n">
+      <x:c r="H4" s="65" t="n">
         <x:f>SUM(C4:F4)</x:f>
         <x:v>231</x:v>
       </x:c>

</xml_diff>